<commit_message>
Fixed Download in DFPD
</commit_message>
<xml_diff>
--- a/pds_admin_Punjab_R/Backend/Backend/Data_3.xlsx
+++ b/pds_admin_Punjab_R/Backend/Backend/Data_3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6733" uniqueCount="2188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6733" uniqueCount="2192">
   <si>
     <t>PC_District</t>
   </si>
@@ -6573,6 +6573,18 @@
   </si>
   <si>
     <t>Remaining_Capacity1</t>
+  </si>
+  <si>
+    <t>Amritsar</t>
+  </si>
+  <si>
+    <t>Fazilka</t>
+  </si>
+  <si>
+    <t>Jalandhar</t>
+  </si>
+  <si>
+    <t>Malerkotla</t>
   </si>
   <si>
     <t>agah</t>
@@ -70522,10 +70534,10 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>2186</v>
       </c>
       <c r="B2" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -70534,7 +70546,7 @@
         <v>31.45335</v>
       </c>
       <c r="E2" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F2">
         <v>74.46541999999999</v>
@@ -70554,10 +70566,10 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>2186</v>
       </c>
       <c r="B3" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -70566,7 +70578,7 @@
         <v>31.8529346</v>
       </c>
       <c r="E3" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F3">
         <v>74.91584450000001</v>
@@ -70586,10 +70598,10 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>2186</v>
       </c>
       <c r="B4" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -70598,7 +70610,7 @@
         <v>31.45335</v>
       </c>
       <c r="E4" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F4">
         <v>74.46541999999999</v>
@@ -70618,10 +70630,10 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>2186</v>
       </c>
       <c r="B5" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -70630,7 +70642,7 @@
         <v>31.800077</v>
       </c>
       <c r="E5" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F5">
         <v>74.588493</v>
@@ -70650,10 +70662,10 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B6" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C6">
         <v>394</v>
@@ -70662,7 +70674,7 @@
         <v>30.08793156</v>
       </c>
       <c r="E6" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F6">
         <v>74.20908439</v>
@@ -70682,10 +70694,10 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B7" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C7">
         <v>395</v>
@@ -70694,7 +70706,7 @@
         <v>30.08675444</v>
       </c>
       <c r="E7" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F7">
         <v>74.20888524</v>
@@ -70714,10 +70726,10 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B8" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C8">
         <v>396</v>
@@ -70726,7 +70738,7 @@
         <v>30.15881226</v>
       </c>
       <c r="E8" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F8">
         <v>74.18214294000001</v>
@@ -70746,10 +70758,10 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B9" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C9">
         <v>397</v>
@@ -70758,7 +70770,7 @@
         <v>30.0974593</v>
       </c>
       <c r="E9" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F9">
         <v>74.206666</v>
@@ -70778,10 +70790,10 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B10" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C10">
         <v>398</v>
@@ -70790,7 +70802,7 @@
         <v>30.15894356</v>
       </c>
       <c r="E10" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F10">
         <v>74.18094151</v>
@@ -70810,10 +70822,10 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B11" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C11">
         <v>399</v>
@@ -70822,7 +70834,7 @@
         <v>30.15848535</v>
       </c>
       <c r="E11" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F11">
         <v>74.18085842000001</v>
@@ -70842,10 +70854,10 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B12" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C12">
         <v>400</v>
@@ -70854,7 +70866,7 @@
         <v>30.15809938</v>
       </c>
       <c r="E12" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F12">
         <v>74.16401603</v>
@@ -70874,10 +70886,10 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B13" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C13">
         <v>401</v>
@@ -70886,7 +70898,7 @@
         <v>30.17081207</v>
       </c>
       <c r="E13" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F13">
         <v>74.18179719</v>
@@ -70906,10 +70918,10 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B14" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C14">
         <v>402</v>
@@ -70918,7 +70930,7 @@
         <v>30.17767461</v>
       </c>
       <c r="E14" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F14">
         <v>74.17723581</v>
@@ -70938,10 +70950,10 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B15" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C15">
         <v>403</v>
@@ -70950,7 +70962,7 @@
         <v>30.1689126</v>
       </c>
       <c r="E15" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F15">
         <v>74.183232</v>
@@ -70970,10 +70982,10 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B16" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C16">
         <v>404</v>
@@ -70982,7 +70994,7 @@
         <v>30.10552983</v>
       </c>
       <c r="E16" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F16">
         <v>74.18014506</v>
@@ -71002,10 +71014,10 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B17" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C17">
         <v>405</v>
@@ -71014,7 +71026,7 @@
         <v>30.15857797</v>
       </c>
       <c r="E17" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F17">
         <v>74.18315728</v>
@@ -71034,10 +71046,10 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B18" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C18">
         <v>406</v>
@@ -71046,7 +71058,7 @@
         <v>30.16991135</v>
       </c>
       <c r="E18" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F18">
         <v>74.18230296</v>
@@ -71066,10 +71078,10 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>2187</v>
       </c>
       <c r="B19" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C19">
         <v>407</v>
@@ -71078,7 +71090,7 @@
         <v>30.126927</v>
       </c>
       <c r="E19" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F19">
         <v>74.161942</v>
@@ -71098,10 +71110,10 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>2188</v>
       </c>
       <c r="B20" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C20">
         <v>625</v>
@@ -71110,7 +71122,7 @@
         <v>31.408658</v>
       </c>
       <c r="E20" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F20">
         <v>75.685958</v>
@@ -71130,10 +71142,10 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B21" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C21">
         <v>864</v>
@@ -71142,7 +71154,7 @@
         <v>30.458388</v>
       </c>
       <c r="E21" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F21">
         <v>74.453514</v>
@@ -71162,10 +71174,10 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B22" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C22">
         <v>865</v>
@@ -71174,7 +71186,7 @@
         <v>30.458388</v>
       </c>
       <c r="E22" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F22">
         <v>74.453514</v>
@@ -71194,10 +71206,10 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B23" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C23">
         <v>866</v>
@@ -71206,7 +71218,7 @@
         <v>30.458388</v>
       </c>
       <c r="E23" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F23">
         <v>74.453514</v>
@@ -71226,10 +71238,10 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B24" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C24">
         <v>867</v>
@@ -71238,7 +71250,7 @@
         <v>30.458388</v>
       </c>
       <c r="E24" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F24">
         <v>74.453514</v>
@@ -71258,10 +71270,10 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B25" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C25">
         <v>868</v>
@@ -71270,7 +71282,7 @@
         <v>30.458388</v>
       </c>
       <c r="E25" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F25">
         <v>74.453514</v>
@@ -71290,10 +71302,10 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B26" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C26">
         <v>869</v>
@@ -71302,7 +71314,7 @@
         <v>30.458388</v>
       </c>
       <c r="E26" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F26">
         <v>74.453514</v>
@@ -71322,10 +71334,10 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B27" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C27">
         <v>870</v>
@@ -71334,7 +71346,7 @@
         <v>30.458388</v>
       </c>
       <c r="E27" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F27">
         <v>74.453514</v>
@@ -71354,10 +71366,10 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B28" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C28">
         <v>871</v>
@@ -71366,7 +71378,7 @@
         <v>30.458388</v>
       </c>
       <c r="E28" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F28">
         <v>74.453514</v>
@@ -71386,10 +71398,10 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B29" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C29">
         <v>872</v>
@@ -71398,7 +71410,7 @@
         <v>30.458388</v>
       </c>
       <c r="E29" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F29">
         <v>74.453514</v>
@@ -71418,10 +71430,10 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B30" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C30">
         <v>873</v>
@@ -71430,7 +71442,7 @@
         <v>30.458388</v>
       </c>
       <c r="E30" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F30">
         <v>74.453514</v>
@@ -71450,10 +71462,10 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B31" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C31">
         <v>874</v>
@@ -71462,7 +71474,7 @@
         <v>30.458388</v>
       </c>
       <c r="E31" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F31">
         <v>74.453514</v>
@@ -71482,10 +71494,10 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B32" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C32">
         <v>875</v>
@@ -71494,7 +71506,7 @@
         <v>30.458388</v>
       </c>
       <c r="E32" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F32">
         <v>74.453514</v>
@@ -71514,10 +71526,10 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B33" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C33">
         <v>876</v>
@@ -71526,7 +71538,7 @@
         <v>30.458388</v>
       </c>
       <c r="E33" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F33">
         <v>74.453514</v>
@@ -71546,10 +71558,10 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B34" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C34">
         <v>877</v>
@@ -71558,7 +71570,7 @@
         <v>30.458388</v>
       </c>
       <c r="E34" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F34">
         <v>74.453514</v>
@@ -71578,10 +71590,10 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B35" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C35">
         <v>878</v>
@@ -71590,7 +71602,7 @@
         <v>30.458388</v>
       </c>
       <c r="E35" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F35">
         <v>74.453514</v>
@@ -71610,10 +71622,10 @@
     </row>
     <row r="36" spans="1:10">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B36" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C36">
         <v>879</v>
@@ -71622,7 +71634,7 @@
         <v>30.458388</v>
       </c>
       <c r="E36" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F36">
         <v>74.453514</v>
@@ -71642,10 +71654,10 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>22</v>
+        <v>2189</v>
       </c>
       <c r="B37" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="C37">
         <v>880</v>
@@ -71654,7 +71666,7 @@
         <v>30.458388</v>
       </c>
       <c r="E37" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="F37">
         <v>74.453514</v>

</xml_diff>

<commit_message>
Updated exe and distance matrix 10/7/2026
</commit_message>
<xml_diff>
--- a/pds_admin_Punjab_R/Backend/Backend/Data_3.xlsx
+++ b/pds_admin_Punjab_R/Backend/Backend/Data_3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6901" uniqueCount="2351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6717" uniqueCount="2347">
   <si>
     <t>PC_District</t>
   </si>
@@ -7056,18 +7056,6 @@
   </si>
   <si>
     <t>Depot</t>
-  </si>
-  <si>
-    <t>verka</t>
-  </si>
-  <si>
-    <t>bhagtanwala</t>
-  </si>
-  <si>
-    <t>chhehrata</t>
-  </si>
-  <si>
-    <t>vallah</t>
   </si>
 </sst>
 </file>
@@ -7480,10 +7468,10 @@
         <v>2175</v>
       </c>
       <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
         <v>431650</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -7538,10 +7526,10 @@
         <v>2175</v>
       </c>
       <c r="H4">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>2788</v>
+        <v>52788</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -7567,10 +7555,10 @@
         <v>2175</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>17750</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -7596,10 +7584,10 @@
         <v>2175</v>
       </c>
       <c r="H6">
-        <v>12425</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>140561.5</v>
+        <v>152986.5</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -7654,10 +7642,10 @@
         <v>2175</v>
       </c>
       <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>98175</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -8118,10 +8106,10 @@
         <v>2178</v>
       </c>
       <c r="H24">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>305214</v>
+        <v>355214</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -8147,10 +8135,10 @@
         <v>2178</v>
       </c>
       <c r="H25">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>25346</v>
+        <v>85346</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -8495,10 +8483,10 @@
         <v>2179</v>
       </c>
       <c r="H37">
-        <v>116111</v>
+        <v>0</v>
       </c>
       <c r="I37">
-        <v>459355</v>
+        <v>575466</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -8553,10 +8541,10 @@
         <v>2179</v>
       </c>
       <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
         <v>88347</v>
-      </c>
-      <c r="I39">
-        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -8611,10 +8599,10 @@
         <v>2179</v>
       </c>
       <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
         <v>11142</v>
-      </c>
-      <c r="I41">
-        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -8698,10 +8686,10 @@
         <v>2180</v>
       </c>
       <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
         <v>35025</v>
-      </c>
-      <c r="I44">
-        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -8727,10 +8715,10 @@
         <v>2180</v>
       </c>
       <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
         <v>52002</v>
-      </c>
-      <c r="I45">
-        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -8756,10 +8744,10 @@
         <v>2180</v>
       </c>
       <c r="H46">
-        <v>320718</v>
+        <v>0</v>
       </c>
       <c r="I46">
-        <v>27472</v>
+        <v>348190</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -8785,10 +8773,10 @@
         <v>2180</v>
       </c>
       <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
         <v>92255</v>
-      </c>
-      <c r="I47">
-        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -9017,10 +9005,10 @@
         <v>2182</v>
       </c>
       <c r="H55">
-        <v>94624.5</v>
+        <v>0</v>
       </c>
       <c r="I55">
-        <v>115466</v>
+        <v>210090.5</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -9046,10 +9034,10 @@
         <v>2182</v>
       </c>
       <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
         <v>17174.5</v>
-      </c>
-      <c r="I56">
-        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -9075,10 +9063,10 @@
         <v>2182</v>
       </c>
       <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
         <v>25993</v>
-      </c>
-      <c r="I57">
-        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -9104,10 +9092,10 @@
         <v>2182</v>
       </c>
       <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
         <v>371327</v>
-      </c>
-      <c r="I58">
-        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -9133,10 +9121,10 @@
         <v>2182</v>
       </c>
       <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
         <v>132901</v>
-      </c>
-      <c r="I59">
-        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -70974,7 +70962,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -71011,31 +70999,31 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>2345</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>394</v>
       </c>
       <c r="D2">
-        <v>31.81488868</v>
+        <v>30.08793156</v>
       </c>
       <c r="E2" t="s">
         <v>2346</v>
       </c>
       <c r="F2">
-        <v>74.76977281000001</v>
+        <v>74.20908439</v>
       </c>
       <c r="G2">
-        <v>160000</v>
+        <v>162900</v>
       </c>
       <c r="H2" t="s">
-        <v>2175</v>
+        <v>2211</v>
       </c>
       <c r="I2">
-        <v>160000</v>
+        <v>162900</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -71043,31 +71031,31 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>2345</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>395</v>
       </c>
       <c r="D3">
-        <v>31.45335</v>
+        <v>30.08675444</v>
       </c>
       <c r="E3" t="s">
         <v>2346</v>
       </c>
       <c r="F3">
-        <v>74.46541999999999</v>
+        <v>74.20888524</v>
       </c>
       <c r="G3">
-        <v>150000</v>
+        <v>53550</v>
       </c>
       <c r="H3" t="s">
-        <v>2175</v>
+        <v>2211</v>
       </c>
       <c r="I3">
-        <v>150000</v>
+        <v>53550</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -71075,31 +71063,31 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>2345</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>396</v>
       </c>
       <c r="D4">
-        <v>31.8529346</v>
+        <v>30.15881226</v>
       </c>
       <c r="E4" t="s">
         <v>2346</v>
       </c>
       <c r="F4">
-        <v>74.91584450000001</v>
+        <v>74.18214294000001</v>
       </c>
       <c r="G4">
-        <v>50000</v>
+        <v>90000</v>
       </c>
       <c r="H4" t="s">
-        <v>2175</v>
+        <v>2211</v>
       </c>
       <c r="I4">
-        <v>50000</v>
+        <v>90000</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -71107,63 +71095,63 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>2345</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>397</v>
       </c>
       <c r="D5">
-        <v>31.45335</v>
+        <v>30.0974593</v>
       </c>
       <c r="E5" t="s">
         <v>2346</v>
       </c>
       <c r="F5">
-        <v>74.46541999999999</v>
+        <v>74.206666</v>
       </c>
       <c r="G5">
-        <v>150000</v>
+        <v>120000</v>
       </c>
       <c r="H5" t="s">
-        <v>2347</v>
+        <v>2211</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="J5">
-        <v>150000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>2345</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>398</v>
       </c>
       <c r="D6">
-        <v>31.800077</v>
+        <v>30.15894356</v>
       </c>
       <c r="E6" t="s">
         <v>2346</v>
       </c>
       <c r="F6">
-        <v>74.588493</v>
+        <v>74.18094151</v>
       </c>
       <c r="G6">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="H6" t="s">
-        <v>2178</v>
+        <v>2211</v>
       </c>
       <c r="I6">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -71171,191 +71159,191 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>2345</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>399</v>
       </c>
       <c r="D7">
-        <v>31.5646079</v>
+        <v>30.15848535</v>
       </c>
       <c r="E7" t="s">
         <v>2346</v>
       </c>
       <c r="F7">
-        <v>74.8878672</v>
+        <v>74.18085842000001</v>
       </c>
       <c r="G7">
-        <v>70000</v>
+        <v>120000</v>
       </c>
       <c r="H7" t="s">
-        <v>2348</v>
+        <v>2211</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="J7">
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>2345</v>
       </c>
       <c r="C8">
-        <v>7</v>
+        <v>400</v>
       </c>
       <c r="D8">
-        <v>31.580623</v>
+        <v>30.15809938</v>
       </c>
       <c r="E8" t="s">
         <v>2346</v>
       </c>
       <c r="F8">
-        <v>74.8949673</v>
+        <v>74.16401603</v>
       </c>
       <c r="G8">
-        <v>120000</v>
+        <v>403500</v>
       </c>
       <c r="H8" t="s">
-        <v>2348</v>
+        <v>2211</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>403500</v>
       </c>
       <c r="J8">
-        <v>120000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>2345</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>401</v>
       </c>
       <c r="D9">
-        <v>31.582043</v>
+        <v>30.17081207</v>
       </c>
       <c r="E9" t="s">
         <v>2346</v>
       </c>
       <c r="F9">
-        <v>74.8871613</v>
+        <v>74.18179719</v>
       </c>
       <c r="G9">
-        <v>35000</v>
+        <v>210541</v>
       </c>
       <c r="H9" t="s">
-        <v>2348</v>
+        <v>2211</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>210541</v>
       </c>
       <c r="J9">
-        <v>35000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
         <v>2345</v>
       </c>
       <c r="C10">
-        <v>9</v>
+        <v>402</v>
       </c>
       <c r="D10">
-        <v>31.45335</v>
+        <v>30.17767461</v>
       </c>
       <c r="E10" t="s">
         <v>2346</v>
       </c>
       <c r="F10">
-        <v>74.46541999999999</v>
+        <v>74.17723581</v>
       </c>
       <c r="G10">
-        <v>35000</v>
+        <v>76960</v>
       </c>
       <c r="H10" t="s">
-        <v>2348</v>
+        <v>2211</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>76960</v>
       </c>
       <c r="J10">
-        <v>35000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>2345</v>
       </c>
       <c r="C11">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="D11">
-        <v>31.45335</v>
+        <v>30.1689126</v>
       </c>
       <c r="E11" t="s">
         <v>2346</v>
       </c>
       <c r="F11">
-        <v>74.46541999999999</v>
+        <v>74.183232</v>
       </c>
       <c r="G11">
-        <v>60000</v>
+        <v>34300</v>
       </c>
       <c r="H11" t="s">
-        <v>2349</v>
+        <v>2211</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>34300</v>
       </c>
       <c r="J11">
-        <v>60000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>2345</v>
       </c>
       <c r="C12">
-        <v>11</v>
+        <v>404</v>
       </c>
       <c r="D12">
-        <v>31.70219884</v>
+        <v>30.10552983</v>
       </c>
       <c r="E12" t="s">
         <v>2346</v>
       </c>
       <c r="F12">
-        <v>74.68916134</v>
+        <v>74.18014506</v>
       </c>
       <c r="G12">
-        <v>35000</v>
+        <v>93500</v>
       </c>
       <c r="H12" t="s">
-        <v>2178</v>
+        <v>2211</v>
       </c>
       <c r="I12">
-        <v>35000</v>
+        <v>93500</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -71363,31 +71351,31 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>2345</v>
       </c>
       <c r="C13">
-        <v>12</v>
+        <v>405</v>
       </c>
       <c r="D13">
-        <v>31.703294</v>
+        <v>30.15857797</v>
       </c>
       <c r="E13" t="s">
         <v>2346</v>
       </c>
       <c r="F13">
-        <v>74.69096380000001</v>
+        <v>74.18315728</v>
       </c>
       <c r="G13">
-        <v>25000</v>
+        <v>150000</v>
       </c>
       <c r="H13" t="s">
-        <v>2178</v>
+        <v>2211</v>
       </c>
       <c r="I13">
-        <v>25000</v>
+        <v>150000</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -71395,31 +71383,31 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>2345</v>
       </c>
       <c r="C14">
-        <v>13</v>
+        <v>406</v>
       </c>
       <c r="D14">
-        <v>31.56972149</v>
+        <v>30.16991135</v>
       </c>
       <c r="E14" t="s">
         <v>2346</v>
       </c>
       <c r="F14">
-        <v>75.09414523</v>
+        <v>74.18230296</v>
       </c>
       <c r="G14">
-        <v>105000</v>
+        <v>74000</v>
       </c>
       <c r="H14" t="s">
-        <v>2179</v>
+        <v>2211</v>
       </c>
       <c r="I14">
-        <v>105000</v>
+        <v>74000</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -71427,63 +71415,63 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>2345</v>
       </c>
       <c r="C15">
-        <v>14</v>
+        <v>407</v>
       </c>
       <c r="D15">
-        <v>31.45335</v>
+        <v>30.126927</v>
       </c>
       <c r="E15" t="s">
         <v>2346</v>
       </c>
       <c r="F15">
-        <v>74.46541999999999</v>
+        <v>74.161942</v>
       </c>
       <c r="G15">
-        <v>70000</v>
+        <v>718340</v>
       </c>
       <c r="H15" t="s">
-        <v>2179</v>
+        <v>2211</v>
       </c>
       <c r="I15">
-        <v>70000</v>
+        <v>702719</v>
       </c>
       <c r="J15">
-        <v>0</v>
+        <v>15621</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>2345</v>
       </c>
       <c r="C16">
-        <v>15</v>
+        <v>625</v>
       </c>
       <c r="D16">
-        <v>31.70744121</v>
+        <v>31.408658</v>
       </c>
       <c r="E16" t="s">
         <v>2346</v>
       </c>
       <c r="F16">
-        <v>74.92578249</v>
+        <v>75.685958</v>
       </c>
       <c r="G16">
-        <v>180000</v>
+        <v>21500</v>
       </c>
       <c r="H16" t="s">
-        <v>2180</v>
+        <v>2236</v>
       </c>
       <c r="I16">
-        <v>180000</v>
+        <v>21500</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -71491,31 +71479,31 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
         <v>2345</v>
       </c>
       <c r="C17">
-        <v>16</v>
+        <v>864</v>
       </c>
       <c r="D17">
-        <v>31.70744121</v>
+        <v>30.458388</v>
       </c>
       <c r="E17" t="s">
         <v>2346</v>
       </c>
       <c r="F17">
-        <v>74.92578249</v>
+        <v>74.453514</v>
       </c>
       <c r="G17">
-        <v>120000</v>
+        <v>294680</v>
       </c>
       <c r="H17" t="s">
-        <v>2180</v>
+        <v>2265</v>
       </c>
       <c r="I17">
-        <v>120000</v>
+        <v>294680</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -71523,31 +71511,31 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
         <v>2345</v>
       </c>
       <c r="C18">
-        <v>17</v>
+        <v>865</v>
       </c>
       <c r="D18">
-        <v>31.52691932</v>
+        <v>30.458388</v>
       </c>
       <c r="E18" t="s">
         <v>2346</v>
       </c>
       <c r="F18">
-        <v>75.26848901</v>
+        <v>74.453514</v>
       </c>
       <c r="G18">
-        <v>17500</v>
+        <v>16680</v>
       </c>
       <c r="H18" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I18">
-        <v>17500</v>
+        <v>16680</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -71555,31 +71543,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B19" t="s">
         <v>2345</v>
       </c>
       <c r="C19">
-        <v>18</v>
+        <v>866</v>
       </c>
       <c r="D19">
-        <v>31.52693009</v>
+        <v>30.458388</v>
       </c>
       <c r="E19" t="s">
         <v>2346</v>
       </c>
       <c r="F19">
-        <v>75.26852979</v>
+        <v>74.453514</v>
       </c>
       <c r="G19">
-        <v>17500</v>
+        <v>126680</v>
       </c>
       <c r="H19" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I19">
-        <v>17500</v>
+        <v>126680</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -71587,31 +71575,31 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
         <v>2345</v>
       </c>
       <c r="C20">
-        <v>19</v>
+        <v>867</v>
       </c>
       <c r="D20">
-        <v>31.543266</v>
+        <v>30.458388</v>
       </c>
       <c r="E20" t="s">
         <v>2346</v>
       </c>
       <c r="F20">
-        <v>75.21952</v>
+        <v>74.453514</v>
       </c>
       <c r="G20">
-        <v>190000</v>
+        <v>10000</v>
       </c>
       <c r="H20" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I20">
-        <v>190000</v>
+        <v>10000</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -71619,31 +71607,31 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
         <v>2345</v>
       </c>
       <c r="C21">
-        <v>20</v>
+        <v>868</v>
       </c>
       <c r="D21">
-        <v>31.543724</v>
+        <v>30.458388</v>
       </c>
       <c r="E21" t="s">
         <v>2346</v>
       </c>
       <c r="F21">
-        <v>75.21528600000001</v>
+        <v>74.453514</v>
       </c>
       <c r="G21">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="H21" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I21">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -71651,31 +71639,31 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>2345</v>
       </c>
       <c r="C22">
-        <v>21</v>
+        <v>869</v>
       </c>
       <c r="D22">
-        <v>31.6647538</v>
+        <v>30.458388</v>
       </c>
       <c r="E22" t="s">
         <v>2346</v>
       </c>
       <c r="F22">
-        <v>75.234335</v>
+        <v>74.453514</v>
       </c>
       <c r="G22">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="H22" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I22">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -71683,63 +71671,63 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>2345</v>
       </c>
       <c r="C23">
-        <v>22</v>
+        <v>870</v>
       </c>
       <c r="D23">
-        <v>31.6603418</v>
+        <v>30.458388</v>
       </c>
       <c r="E23" t="s">
         <v>2346</v>
       </c>
       <c r="F23">
-        <v>74.78764959999999</v>
+        <v>74.453514</v>
       </c>
       <c r="G23">
-        <v>130000</v>
+        <v>10000</v>
       </c>
       <c r="H23" t="s">
-        <v>2347</v>
+        <v>2265</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="J23">
-        <v>130000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>2345</v>
       </c>
       <c r="C24">
-        <v>23</v>
+        <v>871</v>
       </c>
       <c r="D24">
-        <v>31.781936</v>
+        <v>30.458388</v>
       </c>
       <c r="E24" t="s">
         <v>2346</v>
       </c>
       <c r="F24">
-        <v>74.76758049999999</v>
+        <v>74.453514</v>
       </c>
       <c r="G24">
-        <v>250000</v>
+        <v>30720</v>
       </c>
       <c r="H24" t="s">
-        <v>2175</v>
+        <v>2265</v>
       </c>
       <c r="I24">
-        <v>250000</v>
+        <v>30720</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -71747,127 +71735,127 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>2345</v>
       </c>
       <c r="C25">
-        <v>24</v>
+        <v>872</v>
       </c>
       <c r="D25">
-        <v>31.60898</v>
+        <v>30.458388</v>
       </c>
       <c r="E25" t="s">
         <v>2346</v>
       </c>
       <c r="F25">
-        <v>74.78771999999999</v>
+        <v>74.453514</v>
       </c>
       <c r="G25">
-        <v>60000</v>
+        <v>30720</v>
       </c>
       <c r="H25" t="s">
-        <v>2349</v>
+        <v>2265</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>30720</v>
       </c>
       <c r="J25">
-        <v>60000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
         <v>2345</v>
       </c>
       <c r="C26">
-        <v>25</v>
+        <v>873</v>
       </c>
       <c r="D26">
-        <v>31.60898</v>
+        <v>30.458388</v>
       </c>
       <c r="E26" t="s">
         <v>2346</v>
       </c>
       <c r="F26">
-        <v>74.78771999999999</v>
+        <v>74.453514</v>
       </c>
       <c r="G26">
-        <v>80000</v>
+        <v>29640</v>
       </c>
       <c r="H26" t="s">
-        <v>2349</v>
+        <v>2265</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>29640</v>
       </c>
       <c r="J26">
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B27" t="s">
         <v>2345</v>
       </c>
       <c r="C27">
-        <v>26</v>
+        <v>874</v>
       </c>
       <c r="D27">
-        <v>31.598156</v>
+        <v>30.458388</v>
       </c>
       <c r="E27" t="s">
         <v>2346</v>
       </c>
       <c r="F27">
-        <v>74.784094</v>
+        <v>74.453514</v>
       </c>
       <c r="G27">
-        <v>80000</v>
+        <v>28460</v>
       </c>
       <c r="H27" t="s">
-        <v>2349</v>
+        <v>2265</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>28460</v>
       </c>
       <c r="J27">
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B28" t="s">
         <v>2345</v>
       </c>
       <c r="C28">
-        <v>27</v>
+        <v>875</v>
       </c>
       <c r="D28">
-        <v>31.539066</v>
+        <v>30.458388</v>
       </c>
       <c r="E28" t="s">
         <v>2346</v>
       </c>
       <c r="F28">
-        <v>75.244698</v>
+        <v>74.453514</v>
       </c>
       <c r="G28">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="H28" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I28">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="J28">
         <v>0</v>
@@ -71875,31 +71863,31 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B29" t="s">
         <v>2345</v>
       </c>
       <c r="C29">
-        <v>28</v>
+        <v>876</v>
       </c>
       <c r="D29">
-        <v>31.539066</v>
+        <v>30.458388</v>
       </c>
       <c r="E29" t="s">
         <v>2346</v>
       </c>
       <c r="F29">
-        <v>75.244698</v>
+        <v>74.453514</v>
       </c>
       <c r="G29">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="H29" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I29">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -71907,31 +71895,31 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
         <v>2345</v>
       </c>
       <c r="C30">
-        <v>29</v>
+        <v>877</v>
       </c>
       <c r="D30">
-        <v>31.561626</v>
+        <v>30.458388</v>
       </c>
       <c r="E30" t="s">
         <v>2346</v>
       </c>
       <c r="F30">
-        <v>75.140022</v>
+        <v>74.453514</v>
       </c>
       <c r="G30">
-        <v>75000</v>
+        <v>20480</v>
       </c>
       <c r="H30" t="s">
-        <v>2182</v>
+        <v>2265</v>
       </c>
       <c r="I30">
-        <v>75000</v>
+        <v>20480</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -71939,31 +71927,31 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B31" t="s">
         <v>2345</v>
       </c>
       <c r="C31">
-        <v>30</v>
+        <v>878</v>
       </c>
       <c r="D31">
-        <v>31.571434</v>
+        <v>30.458388</v>
       </c>
       <c r="E31" t="s">
         <v>2346</v>
       </c>
       <c r="F31">
-        <v>75.048013</v>
+        <v>74.453514</v>
       </c>
       <c r="G31">
-        <v>25000</v>
+        <v>20480</v>
       </c>
       <c r="H31" t="s">
-        <v>2179</v>
+        <v>2265</v>
       </c>
       <c r="I31">
-        <v>25000</v>
+        <v>20480</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -71971,31 +71959,31 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B32" t="s">
         <v>2345</v>
       </c>
       <c r="C32">
-        <v>31</v>
+        <v>879</v>
       </c>
       <c r="D32">
-        <v>31.583519</v>
+        <v>30.458388</v>
       </c>
       <c r="E32" t="s">
         <v>2346</v>
       </c>
       <c r="F32">
-        <v>75.049741</v>
+        <v>74.453514</v>
       </c>
       <c r="G32">
-        <v>10500</v>
+        <v>20480</v>
       </c>
       <c r="H32" t="s">
-        <v>2179</v>
+        <v>2265</v>
       </c>
       <c r="I32">
-        <v>10500</v>
+        <v>20480</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -72003,1505 +71991,33 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B33" t="s">
         <v>2345</v>
       </c>
       <c r="C33">
-        <v>32</v>
+        <v>880</v>
       </c>
       <c r="D33">
-        <v>31.61865</v>
+        <v>30.458388</v>
       </c>
       <c r="E33" t="s">
         <v>2346</v>
       </c>
       <c r="F33">
-        <v>75.173281</v>
+        <v>74.453514</v>
       </c>
       <c r="G33">
-        <v>65000</v>
+        <v>15360</v>
       </c>
       <c r="H33" t="s">
-        <v>2349</v>
+        <v>2265</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>15360</v>
       </c>
       <c r="J33">
-        <v>65000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10">
-      <c r="A34" t="s">
-        <v>9</v>
-      </c>
-      <c r="B34" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C34">
-        <v>33</v>
-      </c>
-      <c r="D34">
-        <v>31.3844</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F34">
-        <v>75.55336</v>
-      </c>
-      <c r="G34">
-        <v>65710</v>
-      </c>
-      <c r="H34" t="s">
-        <v>2350</v>
-      </c>
-      <c r="I34">
-        <v>0</v>
-      </c>
-      <c r="J34">
-        <v>65710</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10">
-      <c r="A35" t="s">
-        <v>9</v>
-      </c>
-      <c r="B35" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C35">
-        <v>34</v>
-      </c>
-      <c r="D35">
-        <v>31.34177</v>
-      </c>
-      <c r="E35" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F35">
-        <v>75.02247</v>
-      </c>
-      <c r="G35">
-        <v>5100</v>
-      </c>
-      <c r="H35" t="s">
-        <v>2179</v>
-      </c>
-      <c r="I35">
-        <v>5100</v>
-      </c>
-      <c r="J35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10">
-      <c r="A36" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C36">
-        <v>35</v>
-      </c>
-      <c r="D36">
-        <v>31.55489</v>
-      </c>
-      <c r="E36" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F36">
-        <v>75.18541999999999</v>
-      </c>
-      <c r="G36">
-        <v>7070</v>
-      </c>
-      <c r="H36" t="s">
-        <v>2182</v>
-      </c>
-      <c r="I36">
-        <v>7070</v>
-      </c>
-      <c r="J36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
-      <c r="A37" t="s">
-        <v>9</v>
-      </c>
-      <c r="B37" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C37">
-        <v>36</v>
-      </c>
-      <c r="D37">
-        <v>31.5547</v>
-      </c>
-      <c r="E37" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F37">
-        <v>75.18429</v>
-      </c>
-      <c r="G37">
-        <v>17870</v>
-      </c>
-      <c r="H37" t="s">
-        <v>2182</v>
-      </c>
-      <c r="I37">
-        <v>17870</v>
-      </c>
-      <c r="J37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10">
-      <c r="A38" t="s">
-        <v>9</v>
-      </c>
-      <c r="B38" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C38">
-        <v>37</v>
-      </c>
-      <c r="D38">
-        <v>31.5547</v>
-      </c>
-      <c r="E38" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F38">
-        <v>75.18429</v>
-      </c>
-      <c r="G38">
-        <v>130080</v>
-      </c>
-      <c r="H38" t="s">
-        <v>2182</v>
-      </c>
-      <c r="I38">
-        <v>130080</v>
-      </c>
-      <c r="J38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10">
-      <c r="A39" t="s">
-        <v>9</v>
-      </c>
-      <c r="B39" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C39">
-        <v>38</v>
-      </c>
-      <c r="D39">
-        <v>31.43316</v>
-      </c>
-      <c r="E39" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F39">
-        <v>75.00457</v>
-      </c>
-      <c r="G39">
-        <v>100000</v>
-      </c>
-      <c r="H39" t="s">
-        <v>2180</v>
-      </c>
-      <c r="I39">
-        <v>100000</v>
-      </c>
-      <c r="J39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10">
-      <c r="A40" t="s">
-        <v>9</v>
-      </c>
-      <c r="B40" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C40">
-        <v>39</v>
-      </c>
-      <c r="D40">
-        <v>31.43316</v>
-      </c>
-      <c r="E40" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F40">
-        <v>75.00457</v>
-      </c>
-      <c r="G40">
-        <v>50000</v>
-      </c>
-      <c r="H40" t="s">
-        <v>2180</v>
-      </c>
-      <c r="I40">
-        <v>50000</v>
-      </c>
-      <c r="J40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10">
-      <c r="A41" t="s">
-        <v>9</v>
-      </c>
-      <c r="B41" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C41">
-        <v>40</v>
-      </c>
-      <c r="D41">
-        <v>31.43316</v>
-      </c>
-      <c r="E41" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F41">
-        <v>75.00457</v>
-      </c>
-      <c r="G41">
-        <v>125000</v>
-      </c>
-      <c r="H41" t="s">
-        <v>2350</v>
-      </c>
-      <c r="I41">
-        <v>0</v>
-      </c>
-      <c r="J41">
-        <v>125000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10">
-      <c r="A42" t="s">
-        <v>9</v>
-      </c>
-      <c r="B42" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C42">
-        <v>41</v>
-      </c>
-      <c r="D42">
-        <v>31.57114</v>
-      </c>
-      <c r="E42" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F42">
-        <v>74.8843</v>
-      </c>
-      <c r="G42">
-        <v>60000</v>
-      </c>
-      <c r="H42" t="s">
-        <v>2348</v>
-      </c>
-      <c r="I42">
-        <v>0</v>
-      </c>
-      <c r="J42">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10">
-      <c r="A43" t="s">
-        <v>9</v>
-      </c>
-      <c r="B43" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C43">
-        <v>42</v>
-      </c>
-      <c r="D43">
-        <v>31.64602</v>
-      </c>
-      <c r="E43" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F43">
-        <v>74.85684000000001</v>
-      </c>
-      <c r="G43">
-        <v>100000</v>
-      </c>
-      <c r="H43" t="s">
-        <v>2348</v>
-      </c>
-      <c r="I43">
-        <v>0</v>
-      </c>
-      <c r="J43">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10">
-      <c r="A44" t="s">
-        <v>9</v>
-      </c>
-      <c r="B44" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C44">
-        <v>43</v>
-      </c>
-      <c r="D44">
-        <v>31.53422</v>
-      </c>
-      <c r="E44" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F44">
-        <v>75.2328</v>
-      </c>
-      <c r="G44">
-        <v>10000</v>
-      </c>
-      <c r="H44" t="s">
-        <v>2182</v>
-      </c>
-      <c r="I44">
-        <v>10000</v>
-      </c>
-      <c r="J44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10">
-      <c r="A45" t="s">
-        <v>9</v>
-      </c>
-      <c r="B45" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C45">
-        <v>44</v>
-      </c>
-      <c r="D45">
-        <v>31.51572</v>
-      </c>
-      <c r="E45" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F45">
-        <v>75.28874</v>
-      </c>
-      <c r="G45">
-        <v>12000</v>
-      </c>
-      <c r="H45" t="s">
-        <v>2182</v>
-      </c>
-      <c r="I45">
-        <v>12000</v>
-      </c>
-      <c r="J45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10">
-      <c r="A46" t="s">
-        <v>9</v>
-      </c>
-      <c r="B46" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C46">
-        <v>45</v>
-      </c>
-      <c r="D46">
-        <v>31.48214</v>
-      </c>
-      <c r="E46" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F46">
-        <v>74.55329999999999</v>
-      </c>
-      <c r="G46">
-        <v>25000</v>
-      </c>
-      <c r="H46" t="s">
-        <v>2180</v>
-      </c>
-      <c r="I46">
-        <v>25000</v>
-      </c>
-      <c r="J46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10">
-      <c r="A47" t="s">
-        <v>9</v>
-      </c>
-      <c r="B47" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C47">
-        <v>46</v>
-      </c>
-      <c r="D47">
-        <v>31.48214</v>
-      </c>
-      <c r="E47" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F47">
-        <v>74.55329999999999</v>
-      </c>
-      <c r="G47">
-        <v>25000</v>
-      </c>
-      <c r="H47" t="s">
-        <v>2180</v>
-      </c>
-      <c r="I47">
-        <v>25000</v>
-      </c>
-      <c r="J47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10">
-      <c r="A48" t="s">
-        <v>14</v>
-      </c>
-      <c r="B48" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C48">
-        <v>394</v>
-      </c>
-      <c r="D48">
-        <v>30.08793156</v>
-      </c>
-      <c r="E48" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F48">
-        <v>74.20908439</v>
-      </c>
-      <c r="G48">
-        <v>162900</v>
-      </c>
-      <c r="H48" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I48">
-        <v>162900</v>
-      </c>
-      <c r="J48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10">
-      <c r="A49" t="s">
-        <v>14</v>
-      </c>
-      <c r="B49" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C49">
-        <v>395</v>
-      </c>
-      <c r="D49">
-        <v>30.08675444</v>
-      </c>
-      <c r="E49" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F49">
-        <v>74.20888524</v>
-      </c>
-      <c r="G49">
-        <v>53550</v>
-      </c>
-      <c r="H49" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I49">
-        <v>53550</v>
-      </c>
-      <c r="J49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10">
-      <c r="A50" t="s">
-        <v>14</v>
-      </c>
-      <c r="B50" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C50">
-        <v>396</v>
-      </c>
-      <c r="D50">
-        <v>30.15881226</v>
-      </c>
-      <c r="E50" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F50">
-        <v>74.18214294000001</v>
-      </c>
-      <c r="G50">
-        <v>90000</v>
-      </c>
-      <c r="H50" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I50">
-        <v>90000</v>
-      </c>
-      <c r="J50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" t="s">
-        <v>14</v>
-      </c>
-      <c r="B51" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C51">
-        <v>397</v>
-      </c>
-      <c r="D51">
-        <v>30.0974593</v>
-      </c>
-      <c r="E51" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F51">
-        <v>74.206666</v>
-      </c>
-      <c r="G51">
-        <v>120000</v>
-      </c>
-      <c r="H51" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I51">
-        <v>120000</v>
-      </c>
-      <c r="J51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10">
-      <c r="A52" t="s">
-        <v>14</v>
-      </c>
-      <c r="B52" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C52">
-        <v>398</v>
-      </c>
-      <c r="D52">
-        <v>30.15894356</v>
-      </c>
-      <c r="E52" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F52">
-        <v>74.18094151</v>
-      </c>
-      <c r="G52">
-        <v>60000</v>
-      </c>
-      <c r="H52" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I52">
-        <v>60000</v>
-      </c>
-      <c r="J52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10">
-      <c r="A53" t="s">
-        <v>14</v>
-      </c>
-      <c r="B53" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C53">
-        <v>399</v>
-      </c>
-      <c r="D53">
-        <v>30.15848535</v>
-      </c>
-      <c r="E53" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F53">
-        <v>74.18085842000001</v>
-      </c>
-      <c r="G53">
-        <v>120000</v>
-      </c>
-      <c r="H53" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I53">
-        <v>120000</v>
-      </c>
-      <c r="J53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10">
-      <c r="A54" t="s">
-        <v>14</v>
-      </c>
-      <c r="B54" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C54">
-        <v>400</v>
-      </c>
-      <c r="D54">
-        <v>30.15809938</v>
-      </c>
-      <c r="E54" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F54">
-        <v>74.16401603</v>
-      </c>
-      <c r="G54">
-        <v>403500</v>
-      </c>
-      <c r="H54" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I54">
-        <v>403500</v>
-      </c>
-      <c r="J54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10">
-      <c r="A55" t="s">
-        <v>14</v>
-      </c>
-      <c r="B55" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C55">
-        <v>401</v>
-      </c>
-      <c r="D55">
-        <v>30.17081207</v>
-      </c>
-      <c r="E55" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F55">
-        <v>74.18179719</v>
-      </c>
-      <c r="G55">
-        <v>210541</v>
-      </c>
-      <c r="H55" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I55">
-        <v>210541</v>
-      </c>
-      <c r="J55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10">
-      <c r="A56" t="s">
-        <v>14</v>
-      </c>
-      <c r="B56" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C56">
-        <v>402</v>
-      </c>
-      <c r="D56">
-        <v>30.17767461</v>
-      </c>
-      <c r="E56" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F56">
-        <v>74.17723581</v>
-      </c>
-      <c r="G56">
-        <v>76960</v>
-      </c>
-      <c r="H56" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I56">
-        <v>76960</v>
-      </c>
-      <c r="J56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10">
-      <c r="A57" t="s">
-        <v>14</v>
-      </c>
-      <c r="B57" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C57">
-        <v>403</v>
-      </c>
-      <c r="D57">
-        <v>30.1689126</v>
-      </c>
-      <c r="E57" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F57">
-        <v>74.183232</v>
-      </c>
-      <c r="G57">
-        <v>34300</v>
-      </c>
-      <c r="H57" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I57">
-        <v>34300</v>
-      </c>
-      <c r="J57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
-      <c r="A58" t="s">
-        <v>14</v>
-      </c>
-      <c r="B58" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C58">
-        <v>404</v>
-      </c>
-      <c r="D58">
-        <v>30.10552983</v>
-      </c>
-      <c r="E58" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F58">
-        <v>74.18014506</v>
-      </c>
-      <c r="G58">
-        <v>93500</v>
-      </c>
-      <c r="H58" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I58">
-        <v>93500</v>
-      </c>
-      <c r="J58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10">
-      <c r="A59" t="s">
-        <v>14</v>
-      </c>
-      <c r="B59" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C59">
-        <v>405</v>
-      </c>
-      <c r="D59">
-        <v>30.15857797</v>
-      </c>
-      <c r="E59" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F59">
-        <v>74.18315728</v>
-      </c>
-      <c r="G59">
-        <v>150000</v>
-      </c>
-      <c r="H59" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I59">
-        <v>150000</v>
-      </c>
-      <c r="J59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
-      <c r="A60" t="s">
-        <v>14</v>
-      </c>
-      <c r="B60" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C60">
-        <v>406</v>
-      </c>
-      <c r="D60">
-        <v>30.16991135</v>
-      </c>
-      <c r="E60" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F60">
-        <v>74.18230296</v>
-      </c>
-      <c r="G60">
-        <v>74000</v>
-      </c>
-      <c r="H60" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I60">
-        <v>74000</v>
-      </c>
-      <c r="J60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10">
-      <c r="A61" t="s">
-        <v>14</v>
-      </c>
-      <c r="B61" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C61">
-        <v>407</v>
-      </c>
-      <c r="D61">
-        <v>30.126927</v>
-      </c>
-      <c r="E61" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F61">
-        <v>74.161942</v>
-      </c>
-      <c r="G61">
-        <v>718340</v>
-      </c>
-      <c r="H61" t="s">
-        <v>2211</v>
-      </c>
-      <c r="I61">
-        <v>702719</v>
-      </c>
-      <c r="J61">
-        <v>15621</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10">
-      <c r="A62" t="s">
-        <v>18</v>
-      </c>
-      <c r="B62" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C62">
-        <v>625</v>
-      </c>
-      <c r="D62">
-        <v>31.408658</v>
-      </c>
-      <c r="E62" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F62">
-        <v>75.685958</v>
-      </c>
-      <c r="G62">
-        <v>21500</v>
-      </c>
-      <c r="H62" t="s">
-        <v>2236</v>
-      </c>
-      <c r="I62">
-        <v>21500</v>
-      </c>
-      <c r="J62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10">
-      <c r="A63" t="s">
-        <v>22</v>
-      </c>
-      <c r="B63" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C63">
-        <v>864</v>
-      </c>
-      <c r="D63">
-        <v>30.458388</v>
-      </c>
-      <c r="E63" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F63">
-        <v>74.453514</v>
-      </c>
-      <c r="G63">
-        <v>294680</v>
-      </c>
-      <c r="H63" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I63">
-        <v>294680</v>
-      </c>
-      <c r="J63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10">
-      <c r="A64" t="s">
-        <v>22</v>
-      </c>
-      <c r="B64" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C64">
-        <v>865</v>
-      </c>
-      <c r="D64">
-        <v>30.458388</v>
-      </c>
-      <c r="E64" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F64">
-        <v>74.453514</v>
-      </c>
-      <c r="G64">
-        <v>16680</v>
-      </c>
-      <c r="H64" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I64">
-        <v>16680</v>
-      </c>
-      <c r="J64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10">
-      <c r="A65" t="s">
-        <v>22</v>
-      </c>
-      <c r="B65" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C65">
-        <v>866</v>
-      </c>
-      <c r="D65">
-        <v>30.458388</v>
-      </c>
-      <c r="E65" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F65">
-        <v>74.453514</v>
-      </c>
-      <c r="G65">
-        <v>126680</v>
-      </c>
-      <c r="H65" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I65">
-        <v>126680</v>
-      </c>
-      <c r="J65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10">
-      <c r="A66" t="s">
-        <v>22</v>
-      </c>
-      <c r="B66" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C66">
-        <v>867</v>
-      </c>
-      <c r="D66">
-        <v>30.458388</v>
-      </c>
-      <c r="E66" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F66">
-        <v>74.453514</v>
-      </c>
-      <c r="G66">
-        <v>10000</v>
-      </c>
-      <c r="H66" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I66">
-        <v>10000</v>
-      </c>
-      <c r="J66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10">
-      <c r="A67" t="s">
-        <v>22</v>
-      </c>
-      <c r="B67" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C67">
-        <v>868</v>
-      </c>
-      <c r="D67">
-        <v>30.458388</v>
-      </c>
-      <c r="E67" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F67">
-        <v>74.453514</v>
-      </c>
-      <c r="G67">
-        <v>10000</v>
-      </c>
-      <c r="H67" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I67">
-        <v>10000</v>
-      </c>
-      <c r="J67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10">
-      <c r="A68" t="s">
-        <v>22</v>
-      </c>
-      <c r="B68" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C68">
-        <v>869</v>
-      </c>
-      <c r="D68">
-        <v>30.458388</v>
-      </c>
-      <c r="E68" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F68">
-        <v>74.453514</v>
-      </c>
-      <c r="G68">
-        <v>10000</v>
-      </c>
-      <c r="H68" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I68">
-        <v>10000</v>
-      </c>
-      <c r="J68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10">
-      <c r="A69" t="s">
-        <v>22</v>
-      </c>
-      <c r="B69" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C69">
-        <v>870</v>
-      </c>
-      <c r="D69">
-        <v>30.458388</v>
-      </c>
-      <c r="E69" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F69">
-        <v>74.453514</v>
-      </c>
-      <c r="G69">
-        <v>10000</v>
-      </c>
-      <c r="H69" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I69">
-        <v>10000</v>
-      </c>
-      <c r="J69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10">
-      <c r="A70" t="s">
-        <v>22</v>
-      </c>
-      <c r="B70" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C70">
-        <v>871</v>
-      </c>
-      <c r="D70">
-        <v>30.458388</v>
-      </c>
-      <c r="E70" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F70">
-        <v>74.453514</v>
-      </c>
-      <c r="G70">
-        <v>30720</v>
-      </c>
-      <c r="H70" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I70">
-        <v>30720</v>
-      </c>
-      <c r="J70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10">
-      <c r="A71" t="s">
-        <v>22</v>
-      </c>
-      <c r="B71" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C71">
-        <v>872</v>
-      </c>
-      <c r="D71">
-        <v>30.458388</v>
-      </c>
-      <c r="E71" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F71">
-        <v>74.453514</v>
-      </c>
-      <c r="G71">
-        <v>30720</v>
-      </c>
-      <c r="H71" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I71">
-        <v>30720</v>
-      </c>
-      <c r="J71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10">
-      <c r="A72" t="s">
-        <v>22</v>
-      </c>
-      <c r="B72" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C72">
-        <v>873</v>
-      </c>
-      <c r="D72">
-        <v>30.458388</v>
-      </c>
-      <c r="E72" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F72">
-        <v>74.453514</v>
-      </c>
-      <c r="G72">
-        <v>29640</v>
-      </c>
-      <c r="H72" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I72">
-        <v>29640</v>
-      </c>
-      <c r="J72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10">
-      <c r="A73" t="s">
-        <v>22</v>
-      </c>
-      <c r="B73" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C73">
-        <v>874</v>
-      </c>
-      <c r="D73">
-        <v>30.458388</v>
-      </c>
-      <c r="E73" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F73">
-        <v>74.453514</v>
-      </c>
-      <c r="G73">
-        <v>28460</v>
-      </c>
-      <c r="H73" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I73">
-        <v>28460</v>
-      </c>
-      <c r="J73">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10">
-      <c r="A74" t="s">
-        <v>22</v>
-      </c>
-      <c r="B74" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C74">
-        <v>875</v>
-      </c>
-      <c r="D74">
-        <v>30.458388</v>
-      </c>
-      <c r="E74" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F74">
-        <v>74.453514</v>
-      </c>
-      <c r="G74">
-        <v>5000</v>
-      </c>
-      <c r="H74" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I74">
-        <v>5000</v>
-      </c>
-      <c r="J74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10">
-      <c r="A75" t="s">
-        <v>22</v>
-      </c>
-      <c r="B75" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C75">
-        <v>876</v>
-      </c>
-      <c r="D75">
-        <v>30.458388</v>
-      </c>
-      <c r="E75" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F75">
-        <v>74.453514</v>
-      </c>
-      <c r="G75">
-        <v>5000</v>
-      </c>
-      <c r="H75" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I75">
-        <v>5000</v>
-      </c>
-      <c r="J75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10">
-      <c r="A76" t="s">
-        <v>22</v>
-      </c>
-      <c r="B76" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C76">
-        <v>877</v>
-      </c>
-      <c r="D76">
-        <v>30.458388</v>
-      </c>
-      <c r="E76" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F76">
-        <v>74.453514</v>
-      </c>
-      <c r="G76">
-        <v>20480</v>
-      </c>
-      <c r="H76" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I76">
-        <v>20480</v>
-      </c>
-      <c r="J76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10">
-      <c r="A77" t="s">
-        <v>22</v>
-      </c>
-      <c r="B77" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C77">
-        <v>878</v>
-      </c>
-      <c r="D77">
-        <v>30.458388</v>
-      </c>
-      <c r="E77" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F77">
-        <v>74.453514</v>
-      </c>
-      <c r="G77">
-        <v>20480</v>
-      </c>
-      <c r="H77" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I77">
-        <v>20480</v>
-      </c>
-      <c r="J77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10">
-      <c r="A78" t="s">
-        <v>22</v>
-      </c>
-      <c r="B78" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C78">
-        <v>879</v>
-      </c>
-      <c r="D78">
-        <v>30.458388</v>
-      </c>
-      <c r="E78" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F78">
-        <v>74.453514</v>
-      </c>
-      <c r="G78">
-        <v>20480</v>
-      </c>
-      <c r="H78" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I78">
-        <v>20480</v>
-      </c>
-      <c r="J78">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10">
-      <c r="A79" t="s">
-        <v>22</v>
-      </c>
-      <c r="B79" t="s">
-        <v>2345</v>
-      </c>
-      <c r="C79">
-        <v>880</v>
-      </c>
-      <c r="D79">
-        <v>30.458388</v>
-      </c>
-      <c r="E79" t="s">
-        <v>2346</v>
-      </c>
-      <c r="F79">
-        <v>74.453514</v>
-      </c>
-      <c r="G79">
-        <v>15360</v>
-      </c>
-      <c r="H79" t="s">
-        <v>2265</v>
-      </c>
-      <c r="I79">
-        <v>15360</v>
-      </c>
-      <c r="J79">
         <v>0</v>
       </c>
     </row>

</xml_diff>